<commit_message>
Moved JSON generator to a shiny app
</commit_message>
<xml_diff>
--- a/Translation Layer/datasource/APIOntologyModule.xlsx
+++ b/Translation Layer/datasource/APIOntologyModule.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\61084\Desktop\NHDAP Data Lab\ICF Data Lab\GT.Data.Exchange.and.Interoperability\Translation Layer\datasource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085F079B-A5EC-4C5A-9BB8-0F3A7364F89B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E5BCBD-48FC-4A76-B401-CEC8826E1C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DD52E550-EE1D-474D-A99B-0360B6A7F132}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DD52E550-EE1D-474D-A99B-0360B6A7F132}"/>
   </bookViews>
   <sheets>
     <sheet name="Classes" sheetId="1" r:id="rId1"/>
     <sheet name="ClassRelationships" sheetId="2" r:id="rId2"/>
+    <sheet name="Ontology_API Mapping" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="49">
   <si>
     <t>Class</t>
   </si>
@@ -121,6 +122,72 @@
   </si>
   <si>
     <t>includesRequestField</t>
+  </si>
+  <si>
+    <t>OpenAPI Components needed</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Paths</t>
+  </si>
+  <si>
+    <t>/[Class]/[scenario]</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>/client/search</t>
+  </si>
+  <si>
+    <t>InputNeeded</t>
+  </si>
+  <si>
+    <t>InputMapping</t>
+  </si>
+  <si>
+    <t>Path name</t>
+  </si>
+  <si>
+    <t>Operation</t>
+  </si>
+  <si>
+    <t>subclass</t>
+  </si>
+  <si>
+    <t>hasEndpoint owl:get</t>
+  </si>
+  <si>
+    <t>operationId</t>
+  </si>
+  <si>
+    <t>summary</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>requestBody</t>
+  </si>
+  <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>content</t>
+  </si>
+  <si>
+    <t>requestBody/content</t>
+  </si>
+  <si>
+    <t>application/json</t>
+  </si>
+  <si>
+    <t>schema</t>
+  </si>
+  <si>
+    <t>requestBody/content/application/json</t>
   </si>
 </sst>
 </file>
@@ -685,4 +752,121 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3C93419-F17A-4ACA-9E3E-5B4D099BD274}">
+  <dimension ref="A2:D15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>